<commit_message>
Update Q1 FY2027 financials (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -482,7 +482,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-10T10:19:43.497633+00:00</t>
+          <t>2026-07-10T10:19:44.814856+00:00</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-10T10:19:43.497633+00:00</t>
+          <t>2026-07-10T10:19:44.814856+00:00</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-10T10:19:43.497633+00:00</t>
+          <t>2026-07-10T10:19:44.814856+00:00</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-10T10:19:43.497633+00:00</t>
+          <t>2026-07-10T10:19:44.814856+00:00</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-10T10:19:43.497633+00:00</t>
+          <t>2026-07-10T10:19:44.814856+00:00</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-10T10:19:43.497633+00:00</t>
+          <t>2026-07-10T10:19:44.814856+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-10T10:19:43.497633+00:00</t>
+          <t>2026-07-10T10:19:44.814856+00:00</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-10T10:19:43.497633+00:00</t>
+          <t>2026-07-10T10:19:44.814856+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Q2 FY2027 financials (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -717,6 +717,270 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Revenue from Operations</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>200</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:43:19.190333+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>50</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:43:19.190333+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Cost of Materials / COGS</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>80</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:43:19.190333+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Employee Benefit Expense</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:43:19.190333+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Finance Costs</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:43:19.190333+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortization</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>10</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:43:19.190333+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:43:19.190333+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Tax Expense</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>50</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:43:19.190333+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Q3 FY2027 financials (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -981,6 +981,270 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Revenue from Operations</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>150</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:45:44.806363+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>90</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:45:44.806363+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Cost of Materials / COGS</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>50</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:45:44.806363+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Employee Benefit Expense</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>50</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:45:44.806363+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Finance Costs</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:45:44.806363+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortization</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:45:44.806363+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:45:44.806363+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Tax Expense</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:45:44.806363+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Q4 FY2027 financials (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1245,6 +1245,270 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Revenue from Operations</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>400</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:51:00.056150+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>20</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:51:00.056150+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Cost of Materials / COGS</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>80</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:51:00.056150+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Employee Benefit Expense</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:51:00.056150+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Finance Costs</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>4</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:51:00.056150+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortization</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:51:00.056150+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:51:00.056150+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Tax Expense</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>20</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:51:00.056150+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Q4 FY2026 financials (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1509,6 +1509,270 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Revenue from Operations</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>60</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:55:56.280633+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>25</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:55:56.280633+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Cost of Materials / COGS</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>10</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:55:56.280633+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Employee Benefit Expense</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>8</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:55:56.280633+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Finance Costs</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:55:56.280633+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortization</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:55:56.280633+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>15</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:55:56.280633+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Tax Expense</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>20</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-07-10T10:55:56.280633+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Q1 FY2026 financials (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1773,6 +1773,270 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Revenue from Operations</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>60</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-07-13T11:58:43.440801+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-07-13T11:58:43.440801+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Cost of Materials / COGS</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>23</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-07-13T11:58:43.440801+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Employee Benefit Expense</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>9</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-07-13T11:58:43.440801+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Finance Costs</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-07-13T11:58:43.440801+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortization</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-07-13T11:58:43.440801+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-07-13T11:58:43.440801+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Tax Expense</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-07-13T11:58:43.440801+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Q3 FY2026 financials (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2037,6 +2037,270 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Revenue from Operations</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>60.33</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:57:36.442000+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:57:36.442000+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Cost of Materials / COGS</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>8</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:57:36.442000+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Employee Benefit Expense</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:57:36.442000+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Finance Costs</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:57:36.442000+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortization</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>3</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:57:36.442000+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>7</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:57:36.442000+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Tax Expense</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>20.633</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:57:36.442000+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Q2 FY2026 financials (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2301,6 +2301,270 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Revenue from Operations</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>90</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:59:27.962303+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>8</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:59:27.962303+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Cost of Materials / COGS</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>23</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:59:27.962303+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Employee Benefit Expense</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:59:27.962303+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Finance Costs</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:59:27.962303+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortization</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>0.9999</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:59:27.962303+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>22</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:59:27.962303+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Tax Expense</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>23</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2026-07-14T08:59:27.962303+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
AI entry: sold laptops worth 6 lakhs (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1684,6 +1684,92 @@
       <c r="I25" t="inlineStr">
         <is>
           <t>Rejected: I am a bookkeeping assistant designed to record transactions. I do not have access to your historical ledger data to calculate total revenue for a specific period. Please provide specific transaction details if you would like me to record them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-07-16T06:31:22.023698+00:00</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>sold laptops worth 6 lakhs</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Revenue From Operations</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>600000</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-07-16T06:31:22.030809+00:00</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>sold laptops worth 6 lakhs</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Trade Receivables</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>600000</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Applied</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1810,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>30000</v>
+        <v>630000</v>
       </c>
     </row>
     <row r="3">
@@ -1995,7 +2081,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>-20000</v>
+        <v>580000</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
AI entry: purchased office worth 5 crores (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1768,6 +1768,49 @@
         </is>
       </c>
       <c r="I27" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-07-16T06:31:34.959325+00:00</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>purchased office worth 5 crores</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Property, Plant &amp; Equipment</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -2031,7 +2074,7 @@
         </is>
       </c>
       <c r="B3" s="10" t="n">
-        <v>0</v>
+        <v>50000000</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
AI entry: assets purchased 2 lakhs (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1811,6 +1811,92 @@
         </is>
       </c>
       <c r="I28" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-07-16T06:44:23.477315+00:00</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>assets purchased 2 lakhs</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Property, Plant &amp; Equipment</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>200000</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-07-16T06:44:23.484032+00:00</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>assets purchased 2 lakhs</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>200000</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>subtract</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -2598,7 +2684,7 @@
         </is>
       </c>
       <c r="B3" s="10" t="n">
-        <v>0</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="4">
@@ -2658,7 +2744,7 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>-5000000</v>
+        <v>-5200000</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
AI entry: sold goods worth 3 lakhs (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1897,6 +1897,92 @@
         </is>
       </c>
       <c r="I30" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2026-07-18T07:33:21.377357+00:00</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>sold goods worth 3 lakhs</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Revenue From Operations</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>300000</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2026-07-18T07:33:21.383953+00:00</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>sold goods worth 3 lakhs</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>300000</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -1939,7 +2025,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>630000</v>
+        <v>930000</v>
       </c>
     </row>
     <row r="3">
@@ -2220,7 +2306,7 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>-120000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
AI entry: Received interest ₹12,000 (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1983,6 +1983,92 @@
         </is>
       </c>
       <c r="I32" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2026-07-21T04:46:25.293469+00:00</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Received interest ₹12,000</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-07-21T04:46:25.300331+00:00</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Received interest ₹12,000</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -2035,7 +2121,7 @@
         </is>
       </c>
       <c r="B3" s="10" t="n">
-        <v>0</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="4">
@@ -2306,7 +2392,7 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>180000</v>
+        <v>192000</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
AI entry: sold goods worth 20000 (krish)
</commit_message>
<xml_diff>
--- a/data/finance_data.xlsx
+++ b/data/finance_data.xlsx
@@ -15,6 +15,9 @@
     <sheet name="PL_2027_Q2" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="BS_2027_Q2" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="CF_2027_Q2" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="PL_2027_Q3" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="BS_2027_Q3" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="CF_2027_Q3" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -599,13 +602,310 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ASSETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Property, Plant &amp; Equipment</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Right of Use Assets</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Investment Property</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Other Intangible Assets</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Inventories</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Trade Receivables</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>-5180000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Other Current Assets</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TOTAL ASSETS</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>SUM(B3:B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Equity Share Capital</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Other Equity</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LIABILITIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Borrowings</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Trade Payables</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Other Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TOTAL EQUITY &amp; LIABILITIES</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>SUM(B12:B17)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Operating Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Net Cash from Operating</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Investing Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Net Cash from Investing</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Financing Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Net Cash from Financing</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Opening Cash</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Closing Cash</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>SUM(B2,B4,B6,B7)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2069,6 +2369,92 @@
         </is>
       </c>
       <c r="I34" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-07-21T06:51:17.424926+00:00</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>sold goods worth 20000</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Revenue From Operations</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-07-21T06:51:17.430908+00:00</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>sold goods worth 20000</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -3125,4 +3511,213 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Revenue From Operations</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Total Income</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>SUM(B2:B3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cost of Materials Consumed</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Purchases of Stock-in-Trade</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Changes in Inventories</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Employee Benefits Expense</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Finance Costs</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortisation Expenses</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Total Expenses</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>SUM(B7:B13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Profit Before Exceptional Items &amp; Tax</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>B4-B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Exceptional Items</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Profit Before Tax</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>B15-B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Current Tax</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Deferred Tax</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Profit After Tax</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>B17-B18-B19</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>